<commit_message>
Plants: Currant, Sage and Ginseng as general names
The satchel files Desert, Hummingbird and Red Sage as Sage, the two
currants as Currant and the two ginsengs as Ginseng, so those are now
the ingredients, and the plants they are picked from are kept the way
a meat keeps its animals. Oleander Sage stays its own ingredient: only
the poison recipes take it.

- schema 4: plants (id, name, link) and ingredient_plants, from two
  new patch sheets; one row per plant, 33 in all, each for its own
  wiki link
- campfire workbook: recipes and the plant index use the general names
- material dialog and static pages: a Plants section; search finds a
  material by its plants on Materials and Inventory

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/consumable_recipes_rdr2.xlsx
+++ b/data/raw/consumable_recipes_rdr2.xlsx
@@ -785,7 +785,7 @@
 1x Animal Fat</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>[Locked]</t>
         </is>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>1x (Hummingbird Sage / Red Sage / Desert Sage) + 
+          <t>1x Sage + 
 1x Common Bulrush + 
 1x Yarrow</t>
         </is>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>3x (Blackcurrant / Golden Currant) + 
+          <t>3x Currant + 
 3x Beet + 
 3x Hay</t>
         </is>
@@ -1438,7 +1438,7 @@
 1x Moonshine</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>[Locked]</t>
         </is>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>1x (Hummingbird Sage / Red Sage / Desert Sage) + 
+          <t>1x Sage + 
 1x Burdock Root</t>
         </is>
       </c>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>1x (Alaskan Ginseng / American Ginseng) + 
+          <t>1x Ginseng + 
 1x Yarrow</t>
         </is>
       </c>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>1x (Alaskan Ginseng / American Ginseng) + 
+          <t>1x Ginseng + 
 1x Common Bulrush</t>
         </is>
       </c>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>1x (Hummingbird Sage / Red Sage / Desert Sage) + 
+          <t>1x Sage + 
 1x Common Bulrush</t>
         </is>
       </c>
@@ -1837,8 +1837,8 @@
       <c r="D25" s="19" t="inlineStr">
         <is>
           <t>4x Indian Tobacco + 
-4x (Alaskan Ginseng / American Ginseng) + 
-4x (Hummingbird Sage / Red Sage / Desert Sage)</t>
+4x Ginseng + 
+4x Sage</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>2x (Hummingbird Sage / Red Sage / Desert Sage) + 
+          <t>2x Sage + 
 2x Burdock Root + 
 2x (Violet Snowdrop / Wild Feverfew)</t>
         </is>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
-          <t>2x (Alaskan Ginseng / American Ginseng) + 
+          <t>2x Ginseng + 
 2x Yarrow + 
 2x (English Mace / Milkweed)</t>
         </is>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>2x (Alaskan Ginseng / American Ginseng) + 
+          <t>2x Ginseng + 
 2x Common Bulrush + 
 2x Wild Carrot</t>
         </is>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="D33" s="27" t="inlineStr">
         <is>
-          <t>2x (Alaskan Ginseng / American Ginseng) + 
+          <t>2x Ginseng + 
 2x Wild Carrot + 
 2x Parasol Mushroom</t>
         </is>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="D34" s="27" t="inlineStr">
         <is>
-          <t>2x (Hummingbird Sage / Red Sage / Desert Sage) + 
+          <t>2x Sage + 
 2x Common Bulrush + 
 2x Wild Carrot</t>
         </is>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="D35" s="27" t="inlineStr">
         <is>
-          <t>6x (Blackcurrant / Golden Currant) + 
+          <t>6x Currant + 
 6x Yarrow + 
 6x Burdock Root</t>
         </is>
@@ -2394,7 +2394,7 @@
       <c r="D36" s="27" t="inlineStr">
         <is>
           <t>2x Indian Tobacco + 
-2x (Blackcurrant / Golden Currant / Prairie Poppy)</t>
+2x (Currant / Prairie Poppy)</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
@@ -39115,7 +39115,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y34"/>
+  <dimension ref="A1:Y30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="23.13" customWidth="1" style="28" min="1" max="2"/>
@@ -39163,533 +39163,461 @@
       <c r="Y1" s="6" t="n"/>
     </row>
     <row r="2" ht="22.5" customHeight="1" s="28">
-      <c r="A2" s="27">
-        <f> SUBSTITUTE(LOWER(B2), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B2" s="27" t="inlineStr">
-        <is>
-          <t>Alaskan Ginseng</t>
-        </is>
-      </c>
-      <c r="C2" s="18" t="inlineStr">
-        <is>
-          <t>potent-health-cure, potent-horse-medicine, potent-miracle-tonic, special-health-cure, special-horse-medicine, special-horse-reviver</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1" s="28">
-      <c r="A3" s="27">
-        <f> SUBSTITUTE(LOWER(B3), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B3" s="27" t="inlineStr">
-        <is>
-          <t>American Ginseng</t>
-        </is>
-      </c>
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>potent-health-cure, potent-horse-medicine, potent-miracle-tonic, special-health-cure, special-horse-medicine, special-horse-reviver</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1" s="28">
-      <c r="A4" s="27">
+      <c r="A2">
         <f> SUBSTITUTE(LOWER(B4), " ", "-")</f>
         <v/>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Bay Bolete</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>potent-herbivore-bait</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1" s="28">
-      <c r="A5" s="27">
+    <row r="3" ht="22.5" customHeight="1" s="28">
+      <c r="A3">
         <f> SUBSTITUTE(LOWER(B5), " ", "-")</f>
         <v/>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Beet</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>horse-meal</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1" s="28">
-      <c r="A6" s="27">
+    <row r="4" ht="22.5" customHeight="1" s="28">
+      <c r="A4">
         <f> SUBSTITUTE(LOWER(B6), " ", "-")</f>
         <v/>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Blackberry</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>potent-predator-bait, predator-bait</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1" s="28">
-      <c r="A7" s="27">
-        <f> SUBSTITUTE(LOWER(B7), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>Blackcurrant</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>horse-meal, special-miracle-tonic, special-snake-oil</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1" s="28">
-      <c r="A8" s="27">
+    <row r="5" ht="22.5" customHeight="1" s="28">
+      <c r="A5">
         <f> SUBSTITUTE(LOWER(B8), " ", "-")</f>
         <v/>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Burdock Root</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>potent-bitters, special-bitters, special-miracle-tonic</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1" s="28">
-      <c r="A9" s="27">
+    <row r="6" ht="22.5" customHeight="1" s="28">
+      <c r="A6">
         <f> SUBSTITUTE(LOWER(B9), " ", "-")</f>
         <v/>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Chanterelle</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>potent-herbivore-bait</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1" s="28">
-      <c r="A10" s="27">
+    <row r="7" ht="22.5" customHeight="1" s="28">
+      <c r="A7">
         <f> SUBSTITUTE(LOWER(B10), " ", "-")</f>
         <v/>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Common Bulrush</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>horse-ointment, potent-horse-medicine, potent-horse-stimulant, special-horse-medicine, special-horse-stimulant</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1" s="28">
-      <c r="A11" s="27">
+    <row r="8" ht="22.5" customHeight="1" s="28">
+      <c r="A8">
         <f> SUBSTITUTE(LOWER(B11), " ", "-")</f>
         <v/>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Creeping Thyme</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>thyme-big-game, thyme-crustacean, thyme-exotic-bird, thyme-flaky-fish, thyme-game, thyme-mutton, thyme-plump-bird, thyme-pork, thyme-prime-beef, thyme-succulent-fish, thyme-venison</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1" s="28">
-      <c r="A12" s="27">
-        <f> SUBSTITUTE(LOWER(B12), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>Desert Sage</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>horse-ointment, potent-bitters, potent-horse-stimulant, potent-miracle-tonic, special-bitters, special-horse-stimulant</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22.5" customHeight="1" s="28">
-      <c r="A13" s="27">
+    <row r="9" ht="22.5" customHeight="1" s="28">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Currant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>horse-meal, special-miracle-tonic, special-snake-oil</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1" s="28">
+      <c r="A10">
         <f> SUBSTITUTE(LOWER(B13), " ", "-")</f>
         <v/>
       </c>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>English Mace</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>special-health-cure</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1" s="28">
-      <c r="A14" s="27">
+    <row r="11" ht="22.5" customHeight="1" s="28">
+      <c r="A11">
         <f> SUBSTITUTE(LOWER(B14), " ", "-")</f>
         <v/>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Evergreen Huckleberry</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>potent-predator-bait, predator-bait</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1" s="28">
-      <c r="A15" s="27">
-        <f> SUBSTITUTE(LOWER(B15), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Golden Currant</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>horse-meal, special-miracle-tonic, special-snake-oil</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22.5" customHeight="1" s="28">
-      <c r="A16" s="27">
+    <row r="12" ht="22.5" customHeight="1" s="28">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ginseng</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>potent-health-cure, potent-horse-medicine, potent-miracle-tonic, special-health-cure, special-horse-medicine, special-horse-reviver</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1" s="28">
+      <c r="A13">
         <f> SUBSTITUTE(LOWER(B16), " ", "-")</f>
         <v/>
       </c>
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Ground Coffee</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>coffee</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="17.25" customHeight="1" s="28">
-      <c r="A17" s="27">
+    <row r="14" ht="22.5" customHeight="1" s="28">
+      <c r="A14">
         <f> SUBSTITUTE(LOWER(B17), " ", "-")</f>
         <v/>
       </c>
-      <c r="B17" s="27" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Hay</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>horse-meal</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="17.25" customHeight="1" s="28">
-      <c r="A18" s="27">
-        <f> SUBSTITUTE(LOWER(B18), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Hummingbird Sage</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>horse-ointment, potent-bitters, potent-horse-stimulant, potent-miracle-tonic, special-bitters, special-horse-stimulant</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22.5" customHeight="1" s="28">
-      <c r="A19" s="27">
+    <row r="15" ht="22.5" customHeight="1" s="28">
+      <c r="A15">
         <f> SUBSTITUTE(LOWER(B19), " ", "-")</f>
         <v/>
       </c>
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Indian Tobacco</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>potent-miracle-tonic, potent-snake-oil, special-snake-oil</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1" s="28">
-      <c r="A20" s="27">
+    <row r="16" ht="22.5" customHeight="1" s="28">
+      <c r="A16">
         <f> SUBSTITUTE(LOWER(B20), " ", "-")</f>
         <v/>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Milkweed</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>special-health-cure</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1" s="28">
-      <c r="A21" s="27">
+    <row r="17" ht="17.25" customHeight="1" s="28">
+      <c r="A17">
         <f> SUBSTITUTE(LOWER(B21), " ", "-")</f>
         <v/>
       </c>
-      <c r="B21" s="27" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Oleander Sage</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>poison-arrow, poison-throwing-knife</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22.5" customHeight="1" s="28">
-      <c r="A22" s="27">
+    <row r="18" ht="17.25" customHeight="1" s="28">
+      <c r="A18">
         <f> SUBSTITUTE(LOWER(B22), " ", "-")</f>
         <v/>
       </c>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Oregano</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>oregano-big-game, oregano-crustacean, oregano-exotic-bird, oregano-flaky-fish, oregano-game, oregano-mutton, oregano-plump-bird, oregano-pork, oregano-prime-beef, oregano-succulent-fish, oregano-venison</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22.5" customHeight="1" s="28">
-      <c r="A23" s="27">
+    <row r="19" ht="22.5" customHeight="1" s="28">
+      <c r="A19">
         <f> SUBSTITUTE(LOWER(B23), " ", "-")</f>
         <v/>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Parasol Mushroom</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>potent-herbivore-bait, special-horse-reviver</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="22.5" customHeight="1" s="28">
-      <c r="A24" s="27">
+    <row r="20" ht="22.5" customHeight="1" s="28">
+      <c r="A20">
         <f> SUBSTITUTE(LOWER(B24), " ", "-")</f>
         <v/>
       </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Prairie Poppy</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>special-snake-oil</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1" s="28">
-      <c r="A25" s="27">
+    <row r="21" ht="22.5" customHeight="1" s="28">
+      <c r="A21">
         <f> SUBSTITUTE(LOWER(B25), " ", "-")</f>
         <v/>
       </c>
-      <c r="B25" s="27" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Ram's Head</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>potent-herbivore-bait</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1" s="28">
-      <c r="A26" s="27">
+    <row r="22" ht="22.5" customHeight="1" s="28">
+      <c r="A22">
         <f> SUBSTITUTE(LOWER(B26), " ", "-")</f>
         <v/>
       </c>
-      <c r="B26" s="27" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Raspberry</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>potent-predator-bait, predator-bait</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1" s="28">
-      <c r="A27" s="27">
-        <f> SUBSTITUTE(LOWER(B27), " ", "-")</f>
-        <v/>
-      </c>
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t>Red Sage</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="inlineStr">
+    <row r="23" ht="22.5" customHeight="1" s="28">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sage</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>horse-ointment, potent-bitters, potent-horse-stimulant, potent-miracle-tonic, special-bitters, special-horse-stimulant</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22.5" customHeight="1" s="28">
-      <c r="A28" s="27">
+    <row r="24" ht="22.5" customHeight="1" s="28">
+      <c r="A24">
         <f> SUBSTITUTE(LOWER(B28), " ", "-")</f>
         <v/>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Vanilla Flower</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>potent-herbivore-bait</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="22.5" customHeight="1" s="28">
-      <c r="A29" s="27">
+    <row r="25" ht="22.5" customHeight="1" s="28">
+      <c r="A25">
         <f> SUBSTITUTE(LOWER(B29), " ", "-")</f>
         <v/>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Violet Snowdrop</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>potent-herbivore-bait, special-bitters</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22.5" customHeight="1" s="28">
-      <c r="A30" s="27">
+    <row r="26" ht="22.5" customHeight="1" s="28">
+      <c r="A26">
         <f> SUBSTITUTE(LOWER(B30), " ", "-")</f>
         <v/>
       </c>
-      <c r="B30" s="27" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Wild Carrot</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>special-horse-medicine, special-horse-reviver, special-horse-stimulant</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22.5" customHeight="1" s="28">
-      <c r="A31" s="27">
+    <row r="27" ht="22.5" customHeight="1" s="28">
+      <c r="A27">
         <f> SUBSTITUTE(LOWER(B31), " ", "-")</f>
         <v/>
       </c>
-      <c r="B31" s="27" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Wild Feverfew</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>special-bitters</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="22.5" customHeight="1" s="28">
-      <c r="A32" s="27">
+    <row r="28" ht="22.5" customHeight="1" s="28">
+      <c r="A28">
         <f> SUBSTITUTE(LOWER(B32), " ", "-")</f>
         <v/>
       </c>
-      <c r="B32" s="27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Wild Mint</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>minty-big-game, minty-crustacean, minty-exotic-bird, minty-flaky-fish, minty-game, minty-mutton, minty-plump-bird, minty-pork, minty-prime-beef, minty-succulent-fish, minty-venison</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="22.5" customHeight="1" s="28">
-      <c r="A33" s="27">
+    <row r="29" ht="22.5" customHeight="1" s="28">
+      <c r="A29">
         <f> SUBSTITUTE(LOWER(B33), " ", "-")</f>
         <v/>
       </c>
-      <c r="B33" s="27" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Wintergreen Berry</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>potent-predator-bait, predator-bait</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22.5" customHeight="1" s="28">
-      <c r="A34" s="27">
+    <row r="30" ht="22.5" customHeight="1" s="28">
+      <c r="A30">
         <f> SUBSTITUTE(LOWER(B34), " ", "-")</f>
         <v/>
       </c>
-      <c r="B34" s="27" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>Yarrow</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>horse-ointment, potent-health-cure, special-health-cure, special-miracle-tonic</t>
         </is>
       </c>
     </row>
+    <row r="31" ht="22.5" customHeight="1" s="28"/>
+    <row r="32" ht="22.5" customHeight="1" s="28"/>
+    <row r="33" ht="22.5" customHeight="1" s="28"/>
+    <row r="34" ht="22.5" customHeight="1" s="28"/>
     <row r="35" ht="22.5" customHeight="1" s="28"/>
     <row r="36" ht="22.5" customHeight="1" s="28"/>
     <row r="37" ht="22.5" customHeight="1" s="28"/>

</xml_diff>